<commit_message>
SR-11 WIP trying to fix bug in simpleName not falling back to higher level structure and assigning wrong names
</commit_message>
<xml_diff>
--- a/src/main/resources/schema/Mapning genererede tabeller til system_schema_mapping.xlsx
+++ b/src/main/resources/schema/Mapning genererede tabeller til system_schema_mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\R\Desktop\bazaar\src\main\resources\schema\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C5287B81-D2A2-495A-9660-E1E33AC17899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC432095-CCA7-4DFC-B44E-12E496A915BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28800" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{6E07B2F5-6B43-4ECC-99DF-D632EFBC4B65}"/>
+    <workbookView xWindow="11520" yWindow="0" windowWidth="11520" windowHeight="12360" xr2:uid="{6E07B2F5-6B43-4ECC-99DF-D632EFBC4B65}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="53">
   <si>
     <t>gl_entries</t>
   </si>
@@ -144,6 +144,57 @@
   </si>
   <si>
     <t>periodyear</t>
+  </si>
+  <si>
+    <t>recordID</t>
+  </si>
+  <si>
+    <t>accountID</t>
+  </si>
+  <si>
+    <t>analysis</t>
+  </si>
+  <si>
+    <t>valueDate</t>
+  </si>
+  <si>
+    <t>sourceDocumentID</t>
+  </si>
+  <si>
+    <t>customerID</t>
+  </si>
+  <si>
+    <t>supplierID</t>
+  </si>
+  <si>
+    <t>debitAmount</t>
+  </si>
+  <si>
+    <t>creditAmount</t>
+  </si>
+  <si>
+    <t>taxInformation</t>
+  </si>
+  <si>
+    <t>4 = {Attribute@3812} "sourceID: String"</t>
+  </si>
+  <si>
+    <t>5 = {Attribute@3813} "period: BigInteger"</t>
+  </si>
+  <si>
+    <t>6 = {Attribute@3814} "systemID: String"</t>
+  </si>
+  <si>
+    <t>7 = {Attribute@3815} "supplierID: String"</t>
+  </si>
+  <si>
+    <t>8 = {Attribute@3816} "glPostingDate: XMLGregorianCalendar"</t>
+  </si>
+  <si>
+    <t>9 = {Attribute@3817} "systemEntryDate: XMLGregorianCalendar"</t>
+  </si>
+  <si>
+    <t>10 = {Attribute@3818} "Journal_id: Integer"</t>
   </si>
 </sst>
 </file>
@@ -495,18 +546,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B93A043-9E54-4BC6-956B-6F85F4C8353F}">
-  <dimension ref="A1:H24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K33"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1">
         <v>1</v>
       </c>
@@ -529,7 +580,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2</v>
       </c>
@@ -552,7 +603,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>3</v>
       </c>
@@ -575,7 +626,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>4</v>
       </c>
@@ -598,7 +649,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>5</v>
       </c>
@@ -621,7 +672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>6</v>
       </c>
@@ -644,7 +695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>7</v>
       </c>
@@ -667,7 +718,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>8</v>
       </c>
@@ -690,7 +741,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>9</v>
       </c>
@@ -713,7 +764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>10</v>
       </c>
@@ -736,7 +787,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>11</v>
       </c>
@@ -761,8 +812,11 @@
       <c r="H11" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="K11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>12</v>
       </c>
@@ -787,8 +841,15 @@
       <c r="H12" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I12" t="e">
+        <f>+VLOOKUP(F12,$K$11:$K$21,1,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="K12" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>13</v>
       </c>
@@ -813,8 +874,15 @@
       <c r="H13" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I13" t="str">
+        <f t="shared" ref="I13:I24" si="0">+VLOOKUP(F13,$K$11:$K$21,1,FALSE)</f>
+        <v>recordID</v>
+      </c>
+      <c r="K13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>14</v>
       </c>
@@ -839,8 +907,15 @@
       <c r="H14" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I14" t="str">
+        <f t="shared" si="0"/>
+        <v>accountID</v>
+      </c>
+      <c r="K14" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>15</v>
       </c>
@@ -865,8 +940,15 @@
       <c r="H15" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I15" t="str">
+        <f t="shared" si="0"/>
+        <v>supplierID</v>
+      </c>
+      <c r="K15" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>16</v>
       </c>
@@ -891,8 +973,15 @@
       <c r="H16" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I16" t="str">
+        <f t="shared" si="0"/>
+        <v>customerID</v>
+      </c>
+      <c r="K16" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>17</v>
       </c>
@@ -917,8 +1006,15 @@
       <c r="H17" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I17" t="str">
+        <f t="shared" si="0"/>
+        <v>description</v>
+      </c>
+      <c r="K17" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>18</v>
       </c>
@@ -943,8 +1039,15 @@
       <c r="H18" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I18" t="str">
+        <f t="shared" si="0"/>
+        <v>valueDate</v>
+      </c>
+      <c r="K18" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>19</v>
       </c>
@@ -969,8 +1072,15 @@
       <c r="H19" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I19" t="str">
+        <f t="shared" si="0"/>
+        <v>debitAmount</v>
+      </c>
+      <c r="K19" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>20</v>
       </c>
@@ -995,25 +1105,86 @@
       <c r="H20" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I20" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="K20" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="F21" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I21" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+      <c r="K21" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="F22" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I22" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="F23" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I23" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="F24" t="s">
         <v>35</v>
+      </c>
+      <c r="I24" t="e">
+        <f t="shared" si="0"/>
+        <v>#N/A</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G27" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G28" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G29" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G30" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G31" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G32" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="33" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G33" t="s">
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>